<commit_message>
Leadership bios: LinkedIn link on Timothy Vessel and Jessica Cox, as on the source
On highmark.com both bios show the LinkedIn icon, but neither links to a
profile: Timothy Vessel's href is a relative path built from his title, and
Jessica Cox's link has no href. Copied as on the source (decided 2026-10-13):
- import-leadership-bio.js: the importer drops the empty <i class="fab
  fa-linkedin">, so the LinkedIn link is now found as the header's only
  text-less link (besides Request Interview and the PDF) and labelled.
- columns-minimal-dark parser (bio branch): keeps the LinkedIn link whatever
  its href ("#" when it has none).
- scripts.js: decorateLeadershipBio marks header links labelled "LinkedIn"
  with the class linkedin; leadership-bio.css draws the icon for it as well
  as for linkedin.com hrefs.
Re-importing all 16 changes only these two pages (each gains the link).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-leadership-bio.report.xlsx
+++ b/tools/importer/reports/import-leadership-bio.report.xlsx
@@ -1354,7 +1354,7 @@
     <t>leadership-bio</t>
   </si>
   <si>
-    <t>2026-10-12T17:12:09.343Z</t>
+    <t>2026-10-13T13:45:22.504Z</t>
   </si>
   <si>
     <t>Anthony N. Benevento</t>
@@ -1369,7 +1369,7 @@
     <t>about/our-story/leadership-team-board/dan-tropeano</t>
   </si>
   <si>
-    <t>2026-10-12T17:12:34.656Z</t>
+    <t>2026-10-13T13:45:51.231Z</t>
   </si>
   <si>
     <t>Dan Tropeano</t>
@@ -1384,7 +1384,7 @@
     <t>about/our-story/leadership-team-board/david-holmberg</t>
   </si>
   <si>
-    <t>2026-10-12T17:12:39.772Z</t>
+    <t>2026-10-13T13:45:57.760Z</t>
   </si>
   <si>
     <t>David L. Holmberg</t>
@@ -1399,7 +1399,7 @@
     <t>about/our-story/leadership-team-board/edwardshellard</t>
   </si>
   <si>
-    <t>2026-10-12T17:12:03.273Z</t>
+    <t>2026-10-13T13:45:18.355Z</t>
   </si>
   <si>
     <t>Edward Shellard</t>
@@ -1411,7 +1411,7 @@
     <t>about/our-story/leadership-team-board/gustavo-giraldo</t>
   </si>
   <si>
-    <t>2026-10-13T12:06:07.816Z</t>
+    <t>2026-10-13T13:44:50.348Z</t>
   </si>
   <si>
     <t>https://www.highmark.com/about/our-story/leadership-team-board/gustavo-giraldo</t>
@@ -1423,7 +1423,7 @@
     <t>about/our-story/leadership-team-board/jaysheehy</t>
   </si>
   <si>
-    <t>2026-10-13T12:05:55.616Z</t>
+    <t>2026-10-13T13:44:40.879Z</t>
   </si>
   <si>
     <t>https://www.highmark.com/about/our-story/leadership-team-board/JaySheehy</t>
@@ -1435,7 +1435,7 @@
     <t>about/our-story/leadership-team-board/jessicacox</t>
   </si>
   <si>
-    <t>2026-10-13T12:06:18.866Z</t>
+    <t>2026-10-13T13:45:29.170Z</t>
   </si>
   <si>
     <t>https://www.highmark.com/about/our-story/leadership-team-board/JessicaCox</t>
@@ -1447,7 +1447,7 @@
     <t>about/our-story/leadership-team-board/joehaddock</t>
   </si>
   <si>
-    <t>2026-10-12T17:12:25.748Z</t>
+    <t>2026-10-13T13:45:40.476Z</t>
   </si>
   <si>
     <t>Joe Haddock</t>
@@ -1462,7 +1462,7 @@
     <t>about/our-story/leadership-team-board/joy-matoney</t>
   </si>
   <si>
-    <t>2026-10-12T17:11:46.384Z</t>
+    <t>2026-10-13T13:45:02.085Z</t>
   </si>
   <si>
     <t>Joy Matoney</t>
@@ -1477,7 +1477,7 @@
     <t>about/our-story/leadership-team-board/kate-musler</t>
   </si>
   <si>
-    <t>2026-10-13T12:06:13.055Z</t>
+    <t>2026-10-13T13:45:07.627Z</t>
   </si>
   <si>
     <t>https://www.highmark.com/about/our-story/leadership-team-board/kate-musler-</t>
@@ -1489,7 +1489,7 @@
     <t>about/our-story/leadership-team-board/mark-lawrence</t>
   </si>
   <si>
-    <t>2026-10-12T17:11:41.380Z</t>
+    <t>2026-10-13T13:44:55.764Z</t>
   </si>
   <si>
     <t>Mark Lawrence</t>
@@ -1504,7 +1504,7 @@
     <t>about/our-story/leadership-team-board/matthew-rhenish</t>
   </si>
   <si>
-    <t>2026-10-12T17:11:57.133Z</t>
+    <t>2026-10-13T13:45:11.970Z</t>
   </si>
   <si>
     <t>Matthew J. Rhenish</t>
@@ -1519,7 +1519,7 @@
     <t>about/our-story/leadership-team-board/sarah-marche</t>
   </si>
   <si>
-    <t>2026-10-12T17:12:30.408Z</t>
+    <t>2026-10-13T13:45:46.210Z</t>
   </si>
   <si>
     <t>https://www.highmark.com/about/our-story/leadership-team-board/sarah-marche</t>
@@ -1531,7 +1531,7 @@
     <t>about/our-story/leadership-team-board/thomas-fitzpatrick</t>
   </si>
   <si>
-    <t>2026-10-12T17:12:19.485Z</t>
+    <t>2026-10-13T13:45:35.311Z</t>
   </si>
   <si>
     <t>Thomas Fitzpatrick</t>
@@ -1546,7 +1546,7 @@
     <t>about/our-story/leadership-team-board/timothy-vessel</t>
   </si>
   <si>
-    <t>2026-10-13T12:05:49.824Z</t>
+    <t>2026-10-13T13:44:36.218Z</t>
   </si>
   <si>
     <t>Timothy Vessel</t>
@@ -1561,7 +1561,7 @@
     <t>about/our-story/leadership-team-board/victorfields</t>
   </si>
   <si>
-    <t>2026-10-13T12:06:02.363Z</t>
+    <t>2026-10-13T13:44:45.574Z</t>
   </si>
   <si>
     <t>https://www.highmark.com/about/our-story/leadership-team-board/VictorFields</t>

</xml_diff>

<commit_message>
Leadership bios: LinkedIn link on Timothy Vessel and Jessica Cox, as on the source (#100)
On highmark.com both bios show the LinkedIn icon, but neither links to a
profile: Timothy Vessel's href is a relative path built from his title, and
Jessica Cox's link has no href. Copied as on the source (decided 2026-10-13):
- import-leadership-bio.js: the importer drops the empty <i class="fab
  fa-linkedin">, so the LinkedIn link is now found as the header's only
  text-less link (besides Request Interview and the PDF) and labelled.
- columns-minimal-dark parser (bio branch): keeps the LinkedIn link whatever
  its href ("#" when it has none).
- scripts.js: decorateLeadershipBio marks header links labelled "LinkedIn"
  with the class linkedin; leadership-bio.css draws the icon for it as well
  as for linkedin.com hrefs.
Re-importing all 16 changes only these two pages (each gains the link).

Co-authored-by: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-leadership-bio.report.xlsx
+++ b/tools/importer/reports/import-leadership-bio.report.xlsx
@@ -1354,7 +1354,7 @@
     <t>leadership-bio</t>
   </si>
   <si>
-    <t>2026-10-12T17:12:09.343Z</t>
+    <t>2026-10-13T13:45:22.504Z</t>
   </si>
   <si>
     <t>Anthony N. Benevento</t>
@@ -1369,7 +1369,7 @@
     <t>about/our-story/leadership-team-board/dan-tropeano</t>
   </si>
   <si>
-    <t>2026-10-12T17:12:34.656Z</t>
+    <t>2026-10-13T13:45:51.231Z</t>
   </si>
   <si>
     <t>Dan Tropeano</t>
@@ -1384,7 +1384,7 @@
     <t>about/our-story/leadership-team-board/david-holmberg</t>
   </si>
   <si>
-    <t>2026-10-12T17:12:39.772Z</t>
+    <t>2026-10-13T13:45:57.760Z</t>
   </si>
   <si>
     <t>David L. Holmberg</t>
@@ -1399,7 +1399,7 @@
     <t>about/our-story/leadership-team-board/edwardshellard</t>
   </si>
   <si>
-    <t>2026-10-12T17:12:03.273Z</t>
+    <t>2026-10-13T13:45:18.355Z</t>
   </si>
   <si>
     <t>Edward Shellard</t>
@@ -1411,7 +1411,7 @@
     <t>about/our-story/leadership-team-board/gustavo-giraldo</t>
   </si>
   <si>
-    <t>2026-10-13T12:06:07.816Z</t>
+    <t>2026-10-13T13:44:50.348Z</t>
   </si>
   <si>
     <t>https://www.highmark.com/about/our-story/leadership-team-board/gustavo-giraldo</t>
@@ -1423,7 +1423,7 @@
     <t>about/our-story/leadership-team-board/jaysheehy</t>
   </si>
   <si>
-    <t>2026-10-13T12:05:55.616Z</t>
+    <t>2026-10-13T13:44:40.879Z</t>
   </si>
   <si>
     <t>https://www.highmark.com/about/our-story/leadership-team-board/JaySheehy</t>
@@ -1435,7 +1435,7 @@
     <t>about/our-story/leadership-team-board/jessicacox</t>
   </si>
   <si>
-    <t>2026-10-13T12:06:18.866Z</t>
+    <t>2026-10-13T13:45:29.170Z</t>
   </si>
   <si>
     <t>https://www.highmark.com/about/our-story/leadership-team-board/JessicaCox</t>
@@ -1447,7 +1447,7 @@
     <t>about/our-story/leadership-team-board/joehaddock</t>
   </si>
   <si>
-    <t>2026-10-12T17:12:25.748Z</t>
+    <t>2026-10-13T13:45:40.476Z</t>
   </si>
   <si>
     <t>Joe Haddock</t>
@@ -1462,7 +1462,7 @@
     <t>about/our-story/leadership-team-board/joy-matoney</t>
   </si>
   <si>
-    <t>2026-10-12T17:11:46.384Z</t>
+    <t>2026-10-13T13:45:02.085Z</t>
   </si>
   <si>
     <t>Joy Matoney</t>
@@ -1477,7 +1477,7 @@
     <t>about/our-story/leadership-team-board/kate-musler</t>
   </si>
   <si>
-    <t>2026-10-13T12:06:13.055Z</t>
+    <t>2026-10-13T13:45:07.627Z</t>
   </si>
   <si>
     <t>https://www.highmark.com/about/our-story/leadership-team-board/kate-musler-</t>
@@ -1489,7 +1489,7 @@
     <t>about/our-story/leadership-team-board/mark-lawrence</t>
   </si>
   <si>
-    <t>2026-10-12T17:11:41.380Z</t>
+    <t>2026-10-13T13:44:55.764Z</t>
   </si>
   <si>
     <t>Mark Lawrence</t>
@@ -1504,7 +1504,7 @@
     <t>about/our-story/leadership-team-board/matthew-rhenish</t>
   </si>
   <si>
-    <t>2026-10-12T17:11:57.133Z</t>
+    <t>2026-10-13T13:45:11.970Z</t>
   </si>
   <si>
     <t>Matthew J. Rhenish</t>
@@ -1519,7 +1519,7 @@
     <t>about/our-story/leadership-team-board/sarah-marche</t>
   </si>
   <si>
-    <t>2026-10-12T17:12:30.408Z</t>
+    <t>2026-10-13T13:45:46.210Z</t>
   </si>
   <si>
     <t>https://www.highmark.com/about/our-story/leadership-team-board/sarah-marche</t>
@@ -1531,7 +1531,7 @@
     <t>about/our-story/leadership-team-board/thomas-fitzpatrick</t>
   </si>
   <si>
-    <t>2026-10-12T17:12:19.485Z</t>
+    <t>2026-10-13T13:45:35.311Z</t>
   </si>
   <si>
     <t>Thomas Fitzpatrick</t>
@@ -1546,7 +1546,7 @@
     <t>about/our-story/leadership-team-board/timothy-vessel</t>
   </si>
   <si>
-    <t>2026-10-13T12:05:49.824Z</t>
+    <t>2026-10-13T13:44:36.218Z</t>
   </si>
   <si>
     <t>Timothy Vessel</t>
@@ -1561,7 +1561,7 @@
     <t>about/our-story/leadership-team-board/victorfields</t>
   </si>
   <si>
-    <t>2026-10-13T12:06:02.363Z</t>
+    <t>2026-10-13T13:44:45.574Z</t>
   </si>
   <si>
     <t>https://www.highmark.com/about/our-story/leadership-team-board/VictorFields</t>

</xml_diff>